<commit_message>
fix(pcb): connect CH340C to 3V3 instead of 5V, use GPIO5 for TFT_CS, and add extra stiching vias
</commit_message>
<xml_diff>
--- a/hardware/Anemoia-ESP32-SMD/BOM/Bill of Materials-Anemoia-ESP32-SMD.xlsx
+++ b/hardware/Anemoia-ESP32-SMD/BOM/Bill of Materials-Anemoia-ESP32-SMD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\Documents\Altium\Projects\Anemoia-ESP32-SMD\Project Outputs for Anemoia-ESP32-SMD\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9BB036B-B55A-4255-BBF7-F64BE9C561EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C61E44CF-BF5B-43A9-A523-6092203F277E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{3BE75A24-38F2-4C05-A5A1-11986BC0DB6C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{A6725BFF-93FF-4CBE-91AA-16539D5A0D6E}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Anemoia-ESP32" sheetId="1" r:id="rId1"/>
@@ -368,7 +368,7 @@
     <t>RES 10K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>R11, R12, R17, R21, R22, R24, R25, R27, R29, R30, R31</t>
+    <t>R11, R12, R17, R21, R22, R24, R25, R27, R31</t>
   </si>
   <si>
     <t>LTR18EZPJ3R9</t>
@@ -935,7 +935,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EAB41E4-53FB-4A0B-8E96-303341C8410A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E969CD0-1945-4555-A8D3-37DDECE5C32A}">
   <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1480,7 +1480,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>107</v>

</xml_diff>